<commit_message>
Sync tracker + docs with overnight build progress
6 code rows DONE in planning/asset-tracker (xlsx+csv); NEXT_STEPS and
HACKATHON_PLAN note the verified foundation systems and the remaining
real-headset checks.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01398eRPKBRTjBJQ4FDyfbo8
</commit_message>
<xml_diff>
--- a/planning/asset-tracker.xlsx
+++ b/planning/asset-tracker.xlsx
@@ -5426,10 +5426,14 @@
       <c r="K74" s="6" t="inlineStr"/>
       <c r="L74" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="M74" s="6" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="M74" s="6" t="inlineStr">
+        <is>
+          <t>Done overnight; smoke-tested headless.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -5544,10 +5548,14 @@
       <c r="K76" s="6" t="inlineStr"/>
       <c r="L76" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="M76" s="6" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="M76" s="6" t="inlineStr">
+        <is>
+          <t>Done overnight (src/interactions.ts); wave path needs a real-headset check.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -5599,10 +5607,14 @@
       <c r="K77" s="6" t="inlineStr"/>
       <c r="L77" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="M77" s="6" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="M77" s="6" t="inlineStr">
+        <is>
+          <t>Done overnight (src/fade.ts); every teleport now fades. XR quad path needs a headset check.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -5780,10 +5792,14 @@
       <c r="K80" s="6" t="inlineStr"/>
       <c r="L80" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="M80" s="6" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="M80" s="6" t="inlineStr">
+        <is>
+          <t>Done overnight (src/audio.ts); SFX currently 2D — positional attach is a follow-up once real assets land.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
@@ -5839,10 +5855,14 @@
       <c r="K81" s="6" t="inlineStr"/>
       <c r="L81" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="M81" s="6" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="M81" s="6" t="inlineStr">
+        <is>
+          <t>Done overnight.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
@@ -5898,10 +5918,14 @@
       <c r="K82" s="6" t="inlineStr"/>
       <c r="L82" s="6" t="inlineStr">
         <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="M82" s="6" t="inlineStr"/>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="M82" s="6" t="inlineStr">
+        <is>
+          <t>Done overnight (src/companion.ts); billboard live, rigged adapter pending avatar asset.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Sync docs/tracker with avatar-chat companion-mode branch
TECH_SPEC A marked PREPARED (avatar-chat branch claude/webxr-companion-
prompt), NEXT_STEPS deploy note, tracker: backend row updated, cat names
found (Pumpkin, Poppy, Pepper) via the avatar-chat prompt file.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01398eRPKBRTjBJQ4FDyfbo8
</commit_message>
<xml_diff>
--- a/planning/asset-tracker.xlsx
+++ b/planning/asset-tracker.xlsx
@@ -5453,7 +5453,7 @@
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>Backend system_prompt.txt paste (avatar-chat repo)</t>
+          <t>Backend companion mode: deploy to live system_prompt.txt (avatar-chat)</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="I75" s="6" t="inlineStr">
         <is>
-          <t>TECH_SPEC A — paste-ready block: ---TELEPORT:&lt;sceneId&gt;--- marker (BEFORE any ---LINKS---) + companion brevity/guardrails (RAG-grounded, no politics/current events/off-topic, 1-3 spoken sentences). Curl test after restart.</t>
+          <t>PREPARED on avatar-chat branch claude/webxr-companion-prompt: template section (surface-gated so jeffxr.com/chat is untouched), scene_context cap 200-&gt;600 in main.py, 2D marker strip in chat-block.html. Jeff on the Spark: merge branch, copy new section into gitignored system_prompt.txt (keep DYNAMICALLY ADDED KNOWLEDGE), restart jeff-avatar.service, curl test.</t>
         </is>
       </c>
       <c r="J75" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Add cat reference photos + cast the cats; unblock Tripo cat props
Pumpkin (orange tabby), Pepper (gray tabby), Poppy (marbled tabby) —
downscaled reference photos in planning/reference/cats/ with a casting
README. Tracker: cats decision resolved (DONE), the three cat prop rows
now carry coat-accurate image-conditioned prompts (Pepper's sleeping
photo matches the S1 pose exactly; Poppy's sitting photo matches S2),
and the Proxie-with-cats render is logged as an S5 reveal candidate.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01398eRPKBRTjBJQ4FDyfbo8
</commit_message>
<xml_diff>
--- a/planning/asset-tracker.xlsx
+++ b/planning/asset-tracker.xlsx
@@ -869,7 +869,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Cats: names, coat colors, one reference photo each</t>
+          <t>RESOLVED — Cats: Pumpkin (orange tabby), Pepper (gray tabby), Poppy (marbled orange/gray/white tabby); photos in planning/reference/cats/</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
@@ -897,12 +897,12 @@
       <c r="K3" s="6" t="inlineStr"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>NEEDS JEFF</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="M3" s="6" t="inlineStr">
         <is>
-          <t>Blocks 3 Tripo cat props + possibly S5 reveal image.</t>
+          <t>Was blocking 3 Tripo cat props — now unblocked. Cast: Pepper sleeps in S1, Poppy watches the S2 screen, Pumpkin is the S3 hologram.</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>World builder votes cats.</t>
+          <t>World builder votes cats. NEW candidate: the JB Proxie + all-three-cats render (planning/reference/cats/jb-proxie-with-all-three-cats.jpg) — already stylized, Matrix-green sunglasses fit Lightworks; needs grayscale conversion.</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Cat #1 (sleeping)</t>
+          <t>Cat: Pepper, asleep on a crate</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Tripo</t>
+          <t>Tripo (image-conditioned)</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>sleeping cat curled up, short fur, low poly, game ready</t>
+          <t>sleeping gray tabby cat curled up in a tight ball, silver-gray coat with dark charcoal stripes, short fur, game ready</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>Cat decision</t>
+          <t>World gen S1</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="M24" s="6" t="inlineStr">
         <is>
-          <t>BLOCKED on cat decision (names/colors/photos)</t>
+          <t>Image: planning/reference/cats/pepper-gray-tabby-sleeping.jpg (exact pose!); pepper-gray-tabby-alert.jpg for markings</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Cat #2 (watching screen)</t>
+          <t>Cat: Poppy, watching the island game</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>Tripo</t>
+          <t>Tripo (image-conditioned)</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>cat sitting upright on a desk looking at a screen, short fur, low poly, game ready</t>
+          <t>cat sitting upright on a desk looking at a screen, marbled tabby with soft orange gray and white patches, white chest and front paws, short fur, game ready</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>Cat decision</t>
+          <t>World gen S2</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="M34" s="6" t="inlineStr">
         <is>
-          <t>BLOCKED on cat decision</t>
+          <t>Image: planning/reference/cats/poppy-marbled-tabby-sitting.jpg (exact pose)</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Holo-cat #3 (wireframe patrol)</t>
+          <t>Holo-cat: Pumpkin, wireframe patrol</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>low poly cat walking, game ready</t>
+          <t>low poly chunky orange tabby cat walking, rounded belly, game ready</t>
         </is>
       </c>
       <c r="J43" s="6" t="inlineStr">
@@ -3424,7 +3424,7 @@
       </c>
       <c r="K43" s="6" t="inlineStr">
         <is>
-          <t>Cat decision</t>
+          <t>World gen S3</t>
         </is>
       </c>
       <c r="L43" s="6" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="M43" s="6" t="inlineStr">
         <is>
-          <t>BLOCKED on cat decision</t>
+          <t>Wireframe hides color; keep Pumpkin's generous silhouette. Ref: planning/reference/cats/pumpkin-orange-tabby.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S5 reveal image: adopt Jeff's bit-plane decomposition design
Replaces the purely-procedural projector-grid shader with a baked
reconstruction of a real source image (Jeff's Even Realities G2/R1
portrait) via randomized bit-plane decomposition into 4 binary masks
that sum back to a 5-level luminance image -- more faithful to the real
optical all-reduce research and cheaper at runtime than the noise
version (one texture sample + dot product vs. four hash evals). Adds a
click-to-YouTube-review interaction on the resolved screen. Original
procedural shader kept in TECH_SPEC as Plan B fallback.

Tracker: entry scene + reveal image decisions resolved (2 of 7 done),
new bake-script code row, updated prop row. Blocked on the actual source
image landing on disk to run the bake.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01398eRPKBRTjBJQ4FDyfbo8
</commit_message>
<xml_diff>
--- a/planning/asset-tracker.xlsx
+++ b/planning/asset-tracker.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tracker'!$A$1:$M$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tracker'!$A$1:$M$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M94"/>
+  <dimension ref="A1:M95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -814,7 +814,7 @@
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>Entry scene: S1 Hangar (chronological, recommended) or S3 Holo Stage (career-first)?</t>
+          <t>RESOLVED — Entry scene: S1 Hangar (chronological)</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
@@ -842,12 +842,12 @@
       <c r="K2" s="6" t="inlineStr"/>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>NEEDS JEFF</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="M2" s="6" t="inlineStr">
         <is>
-          <t>Blocks defaultSceneId + demo script.</t>
+          <t>Blocks defaultSceneId + demo script. Confirmed 2026-07-19.</t>
         </is>
       </c>
     </row>
@@ -924,7 +924,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>S5 projector-wall reveal image: Jeff portrait / the three cats / logo?</t>
+          <t>RESOLVED — S5 projector-wall reveal image: Even Realities G2/R1 portrait (Louvre pyramid selfie, cropped to remove logo/text/product inset), reconstructed via bit-plane decomposition, click opens youtu.be/sEDTmvGg-QY</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -952,12 +952,12 @@
       <c r="K4" s="6" t="inlineStr"/>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>NEEDS JEFF</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>World builder votes cats. NEW candidate: the JB Proxie + all-three-cats render (planning/reference/cats/jb-proxie-with-all-three-cats.jpg) — already stylized, Matrix-green sunglasses fit Lightworks; needs grayscale conversion.</t>
+          <t>Jeff's design upgrade over the original procedural-noise plan — see TECH_SPEC.md §F. AWAITING: source image file on disk (not yet saved from chat) to run the actual bake script.</t>
         </is>
       </c>
     </row>
@@ -4303,7 +4303,7 @@
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Binary grid textures (x4) + reveal image</t>
+          <t>Baked bit-plane mask texture (reveal image)</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
@@ -4313,7 +4313,7 @@
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>Mint images + custom shader</t>
+          <t>custom bake script (scripts/bake-projector-image.mjs)</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
@@ -4328,12 +4328,12 @@
       </c>
       <c r="I57" s="6" t="inlineStr">
         <is>
-          <t>dense black and white binary square grid pattern, QR-like, flat texture (x4 masks) + 1 grayscale reveal image (PENDING Jeff decision)</t>
+          <t>Source: Jeff's Even Realities G2/R1 review portrait (Louvre pyramid), cropped to remove logo/text/product inset. Bake: downsample to 32x24 cells, quantize to 5 luminance levels, randomly assign which N-of-4 projector channels are on per cell, pack into one RGBA8 PNG (R/G/B/A = projector 0-3 bit). See TECH_SPEC.md §F.</t>
         </is>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
-          <t>Additive-blend light planes summing to reveal (engineer shader).</t>
+          <t>Shader sums the 4 channels via uEnabled dot product (TECH_SPEC F); click on the resolved screen opens youtu.be/sEDTmvGg-QY.</t>
         </is>
       </c>
       <c r="K57" s="6" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="M57" s="6" t="inlineStr">
         <is>
-          <t>Reveal image = open decision</t>
+          <t>AWAITING source image file (Jeff shared inline, not yet saved to a path I can bake from)</t>
         </is>
       </c>
     </row>
@@ -6029,12 +6029,12 @@
       </c>
       <c r="I84" s="6" t="inlineStr">
         <is>
-          <t>TECH_SPEC F — 4 procedural binary grids summed in one fragment shader, 5 brightness steps, beam cones, 4 manifest levers; ~11 draw calls, zero lights.</t>
+          <t>TECH_SPEC F — texture-sum fragment shader (baked bit-plane mask, Plan A) with procedural-noise fallback (Plan B) behind the same uEnabled contract, 5 brightness steps, beam cones, 4 manifest levers; ~11 draw calls, zero lights.</t>
         </is>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>Reveal-image variant needs the Mint textures instead of pure procedural — same shader slot.</t>
+          <t>Click on resolved screen opens youtu.be/sEDTmvGg-QY via the standard interaction.click handler.</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr">
@@ -6062,17 +6062,17 @@
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S5</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>MiniGameSystem RT core (flat-disc MVP)</t>
+          <t>bake-projector-image.mjs script</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>code (5h)</t>
+          <t>code (1h)</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
@@ -6082,22 +6082,22 @@
       </c>
       <c r="G85" s="6" t="inlineStr">
         <is>
-          <t>XR Engineer</t>
+          <t>Blocked on source image file</t>
         </is>
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr">
         <is>
-          <t>TECH_SPEC G — 512px RGBA8 RT at 30Hz, hard pause conditions, xr.enabled save/restore, engage mode suppressing WASD, gaze-UV steering (left/right thirds -&gt; camera CCW/CW), squeeze/pinch/W walk.</t>
+          <t>TECH_SPEC F — Node script: crop/letterbox source image, downsample to 32x24 cells, quantize to 5 luminance levels, randomly assign N-of-4 projector bits per cell (seeded), pack into one RGBA8 PNG.</t>
         </is>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>HOUR-5 CHECKPOINT: playable on flat green disc = feature ships.</t>
+          <t>One-time offline bake, not a runtime system.</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr">
@@ -6130,12 +6130,12 @@
       </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>Mini-game island + character polish</t>
+          <t>MiniGameSystem RT core (flat-disc MVP)</t>
         </is>
       </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
-          <t>code (3-4h)</t>
+          <t>code (5h)</t>
         </is>
       </c>
       <c r="F86" s="6" t="inlineStr">
@@ -6150,17 +6150,17 @@
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
         <is>
-          <t>TECH_SPEC G — island GLB &lt;=20k tris + rigged walker &lt;=10k tris (Tripo P-series 'game ready'), heightfield walk, palm sway optional.</t>
+          <t>TECH_SPEC G — 512px RGBA8 RT at 30Hz, hard pause conditions, xr.enabled save/restore, engage mode suppressing WASD, gaze-UV steering (left/right thirds -&gt; camera CCW/CW), squeeze/pinch/W walk.</t>
         </is>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
-          <t>Assets parallel-track.</t>
+          <t>HOUR-5 CHECKPOINT: playable on flat green disc = feature ships.</t>
         </is>
       </c>
       <c r="K86" s="6" t="inlineStr">
@@ -6193,12 +6193,12 @@
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>Rubber-hand sequence logic</t>
+          <t>Mini-game island + character polish</t>
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t>code (2h)</t>
+          <t>code (3-4h)</t>
         </is>
       </c>
       <c r="F87" s="6" t="inlineStr">
@@ -6213,17 +6213,17 @@
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="I87" s="6" t="inlineStr">
         <is>
-          <t>Stroke-zone counting (N&gt;=5) -&gt; Proxie twitch anim; hammer tap -&gt; flinch+yelp; desktop click auto-stroke.</t>
+          <t>TECH_SPEC G — island GLB &lt;=20k tris + rigged walker &lt;=10k tris (Tripo P-series 'game ready'), heightfield walk, palm sway optional.</t>
         </is>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
-          <t>Needs avatar anim states or mannequin-arm fallback — decide by Sat noon.</t>
+          <t>Assets parallel-track.</t>
         </is>
       </c>
       <c r="K87" s="6" t="inlineStr">
@@ -6251,17 +6251,17 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="D88" s="6" t="inlineStr">
         <is>
-          <t>Server-repair sequence logic</t>
+          <t>Rubber-hand sequence logic</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>code (1.5h)</t>
+          <t>code (2h)</t>
         </is>
       </c>
       <c r="F88" s="6" t="inlineStr">
@@ -6281,10 +6281,14 @@
       </c>
       <c r="I88" s="6" t="inlineStr">
         <is>
-          <t>3-step state machine over interactable events: sled -&gt; faulty out (cart foam) -&gt; replacement in -&gt; aisle LED ripple.</t>
-        </is>
-      </c>
-      <c r="J88" s="6" t="inlineStr"/>
+          <t>Stroke-zone counting (N&gt;=5) -&gt; Proxie twitch anim; hammer tap -&gt; flinch+yelp; desktop click auto-stroke.</t>
+        </is>
+      </c>
+      <c r="J88" s="6" t="inlineStr">
+        <is>
+          <t>Needs avatar anim states or mannequin-arm fallback — decide by Sat noon.</t>
+        </is>
+      </c>
       <c r="K88" s="6" t="inlineStr">
         <is>
           <t>Interactable framework</t>
@@ -6310,17 +6314,17 @@
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S5</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Spline-ribbon drawing</t>
+          <t>Server-repair sequence logic</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>code (2h)</t>
+          <t>code (1.5h)</t>
         </is>
       </c>
       <c r="F89" s="6" t="inlineStr">
@@ -6340,7 +6344,7 @@
       </c>
       <c r="I89" s="6" t="inlineStr">
         <is>
-          <t>Extruded tube along controller/cursor path, capped length, oldest fades; palette detents set color/width.</t>
+          <t>3-step state machine over interactable events: sled -&gt; faulty out (cart foam) -&gt; replacement in -&gt; aisle LED ripple.</t>
         </is>
       </c>
       <c r="J89" s="6" t="inlineStr"/>
@@ -6369,17 +6373,17 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
         <is>
-          <t>Scene anim garnish (windmill sails, Chinook quarter-turn, canopy glow)</t>
+          <t>Spline-ribbon drawing</t>
         </is>
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>code (1.5h)</t>
+          <t>code (2h)</t>
         </is>
       </c>
       <c r="F90" s="6" t="inlineStr">
@@ -6394,12 +6398,12 @@
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="I90" s="6" t="inlineStr">
         <is>
-          <t>Simple rotation/emissive drivers via interactable effects + tiny per-role handlers.</t>
+          <t>Extruded tube along controller/cursor path, capped length, oldest fades; palette detents set color/width.</t>
         </is>
       </c>
       <c r="J90" s="6" t="inlineStr"/>
@@ -6428,12 +6432,12 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Manifest restructure to 5-scene roster + prompts.md population</t>
+          <t>Scene anim garnish (windmill sails, Chinook quarter-turn, canopy glow)</t>
         </is>
       </c>
       <c r="E91" s="6" t="inlineStr">
@@ -6448,25 +6452,25 @@
       </c>
       <c r="G91" s="6" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>XR Engineer</t>
         </is>
       </c>
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr">
         <is>
-          <t>WORLD_DESIGNS roster: worlds roots/career, new sceneIds, portal graph incl. S4 cul-de-sac; migrate placards into props arrays; populate per-scene prompts.md from this tracker.</t>
-        </is>
-      </c>
-      <c r="J91" s="6" t="inlineStr">
-        <is>
-          <t>AFTER Jeff signs off the roster.</t>
-        </is>
-      </c>
-      <c r="K91" s="6" t="inlineStr"/>
+          <t>Simple rotation/emissive drivers via interactable effects + tiny per-role handlers.</t>
+        </is>
+      </c>
+      <c r="J91" s="6" t="inlineStr"/>
+      <c r="K91" s="6" t="inlineStr">
+        <is>
+          <t>Interactable framework</t>
+        </is>
+      </c>
       <c r="L91" s="6" t="inlineStr">
         <is>
           <t>TODO</t>
@@ -6492,12 +6496,12 @@
       </c>
       <c r="D92" s="6" t="inlineStr">
         <is>
-          <t>Portal splat prefetch (fetch-only)</t>
+          <t>Manifest restructure to 5-scene roster + prompts.md population</t>
         </is>
       </c>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>code (1h)</t>
+          <t>code (1.5h)</t>
         </is>
       </c>
       <c r="F92" s="6" t="inlineStr">
@@ -6507,22 +6511,22 @@
       </c>
       <c r="G92" s="6" t="inlineStr">
         <is>
-          <t>XR Engineer</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="I92" s="6" t="inlineStr">
         <is>
-          <t>TECH_SPEC H — warm HTTP cache for entryPortals targets 3s after scene-changed; requestIdleCallback; skip on saveData.</t>
+          <t>WORLD_DESIGNS roster: worlds roots/career, new sceneIds, portal graph incl. S4 cul-de-sac; migrate placards into props arrays; populate per-scene prompts.md from this tracker.</t>
         </is>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>Stretch.</t>
+          <t>AFTER Jeff signs off the roster.</t>
         </is>
       </c>
       <c r="K92" s="6" t="inlineStr"/>
@@ -6551,12 +6555,12 @@
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Quest 3 pass on deployed URL</t>
+          <t>Portal splat prefetch (fetch-only)</t>
         </is>
       </c>
       <c r="E93" s="6" t="inlineStr">
         <is>
-          <t>code (1h x2)</t>
+          <t>code (1h)</t>
         </is>
       </c>
       <c r="F93" s="6" t="inlineStr">
@@ -6571,15 +6575,19 @@
       </c>
       <c r="H93" s="6" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
         <is>
-          <t>TECH_SPEC H test matrix — TTS voices, mic absence, audio unlock, CORS origin, frame budget. End of each build block.</t>
-        </is>
-      </c>
-      <c r="J93" s="6" t="inlineStr"/>
+          <t>TECH_SPEC H — warm HTTP cache for entryPortals targets 3s after scene-changed; requestIdleCallback; skip on saveData.</t>
+        </is>
+      </c>
+      <c r="J93" s="6" t="inlineStr">
+        <is>
+          <t>Stretch.</t>
+        </is>
+      </c>
       <c r="K93" s="6" t="inlineStr"/>
       <c r="L93" s="6" t="inlineStr">
         <is>
@@ -6606,12 +6614,12 @@
       </c>
       <c r="D94" s="6" t="inlineStr">
         <is>
-          <t>Final judging rehearsal (protected)</t>
+          <t>Quest 3 pass on deployed URL</t>
         </is>
       </c>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t>code (2h)</t>
+          <t>code (1h x2)</t>
         </is>
       </c>
       <c r="F94" s="6" t="inlineStr">
@@ -6631,7 +6639,7 @@
       </c>
       <c r="I94" s="6" t="inlineStr">
         <is>
-          <t>Full desktop + Quest walkthrough of demo script; do NOT trade for features.</t>
+          <t>TECH_SPEC H test matrix — TTS voices, mic absence, audio unlock, CORS origin, frame budget. End of each build block.</t>
         </is>
       </c>
       <c r="J94" s="6" t="inlineStr"/>
@@ -6643,8 +6651,63 @@
       </c>
       <c r="M94" s="6" t="inlineStr"/>
     </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>T094</t>
+        </is>
+      </c>
+      <c r="B95" s="11" t="inlineStr">
+        <is>
+          <t>5-Code</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>Final judging rehearsal (protected)</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>code (2h)</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G95" s="6" t="inlineStr">
+        <is>
+          <t>XR Engineer</t>
+        </is>
+      </c>
+      <c r="H95" s="6" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I95" s="6" t="inlineStr">
+        <is>
+          <t>Full desktop + Quest walkthrough of demo script; do NOT trade for features.</t>
+        </is>
+      </c>
+      <c r="J95" s="6" t="inlineStr"/>
+      <c r="K95" s="6" t="inlineStr"/>
+      <c r="L95" s="6" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="M95" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M94"/>
+  <autoFilter ref="A1:M95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6701,11 +6764,11 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>COUNTIF(Tracker!$B$2:$B$94,A5)</f>
+        <f>COUNTIF(Tracker!$B$2:$B$95,A5)</f>
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>COUNTIFS(Tracker!$B$2:$B$94,A5,Tracker!$L$2:$L$94,"DONE")</f>
+        <f>COUNTIFS(Tracker!$B$2:$B$95,A5,Tracker!$L$2:$L$95,"DONE")</f>
         <v/>
       </c>
     </row>
@@ -6716,11 +6779,11 @@
         </is>
       </c>
       <c r="B6" s="3">
-        <f>COUNTIF(Tracker!$B$2:$B$94,A6)</f>
+        <f>COUNTIF(Tracker!$B$2:$B$95,A6)</f>
         <v/>
       </c>
       <c r="C6" s="3">
-        <f>COUNTIFS(Tracker!$B$2:$B$94,A6,Tracker!$L$2:$L$94,"DONE")</f>
+        <f>COUNTIFS(Tracker!$B$2:$B$95,A6,Tracker!$L$2:$L$95,"DONE")</f>
         <v/>
       </c>
     </row>
@@ -6731,11 +6794,11 @@
         </is>
       </c>
       <c r="B7" s="3">
-        <f>COUNTIF(Tracker!$B$2:$B$94,A7)</f>
+        <f>COUNTIF(Tracker!$B$2:$B$95,A7)</f>
         <v/>
       </c>
       <c r="C7" s="3">
-        <f>COUNTIFS(Tracker!$B$2:$B$94,A7,Tracker!$L$2:$L$94,"DONE")</f>
+        <f>COUNTIFS(Tracker!$B$2:$B$95,A7,Tracker!$L$2:$L$95,"DONE")</f>
         <v/>
       </c>
     </row>
@@ -6746,11 +6809,11 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <f>COUNTIF(Tracker!$B$2:$B$94,A8)</f>
+        <f>COUNTIF(Tracker!$B$2:$B$95,A8)</f>
         <v/>
       </c>
       <c r="C8" s="3">
-        <f>COUNTIFS(Tracker!$B$2:$B$94,A8,Tracker!$L$2:$L$94,"DONE")</f>
+        <f>COUNTIFS(Tracker!$B$2:$B$95,A8,Tracker!$L$2:$L$95,"DONE")</f>
         <v/>
       </c>
     </row>
@@ -6761,11 +6824,11 @@
         </is>
       </c>
       <c r="B9" s="3">
-        <f>COUNTIF(Tracker!$B$2:$B$94,A9)</f>
+        <f>COUNTIF(Tracker!$B$2:$B$95,A9)</f>
         <v/>
       </c>
       <c r="C9" s="3">
-        <f>COUNTIFS(Tracker!$B$2:$B$94,A9,Tracker!$L$2:$L$94,"DONE")</f>
+        <f>COUNTIFS(Tracker!$B$2:$B$95,A9,Tracker!$L$2:$L$95,"DONE")</f>
         <v/>
       </c>
     </row>
@@ -6776,11 +6839,11 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>COUNTIF(Tracker!$B$2:$B$94,A10)</f>
+        <f>COUNTIF(Tracker!$B$2:$B$95,A10)</f>
         <v/>
       </c>
       <c r="C10" s="3">
-        <f>COUNTIFS(Tracker!$B$2:$B$94,A10,Tracker!$L$2:$L$94,"DONE")</f>
+        <f>COUNTIFS(Tracker!$B$2:$B$95,A10,Tracker!$L$2:$L$95,"DONE")</f>
         <v/>
       </c>
     </row>
@@ -6810,7 +6873,7 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <f>COUNTIF(Tracker!$L$2:$L$94,A14)</f>
+        <f>COUNTIF(Tracker!$L$2:$L$95,A14)</f>
         <v/>
       </c>
     </row>
@@ -6821,7 +6884,7 @@
         </is>
       </c>
       <c r="B15" s="3">
-        <f>COUNTIF(Tracker!$L$2:$L$94,A15)</f>
+        <f>COUNTIF(Tracker!$L$2:$L$95,A15)</f>
         <v/>
       </c>
     </row>
@@ -6832,7 +6895,7 @@
         </is>
       </c>
       <c r="B16" s="3">
-        <f>COUNTIF(Tracker!$L$2:$L$94,A16)</f>
+        <f>COUNTIF(Tracker!$L$2:$L$95,A16)</f>
         <v/>
       </c>
     </row>
@@ -6843,7 +6906,7 @@
         </is>
       </c>
       <c r="B17" s="3">
-        <f>COUNTIF(Tracker!$L$2:$L$94,A17)</f>
+        <f>COUNTIF(Tracker!$L$2:$L$95,A17)</f>
         <v/>
       </c>
     </row>
@@ -6854,7 +6917,7 @@
         </is>
       </c>
       <c r="B18" s="3">
-        <f>COUNTIF(Tracker!$L$2:$L$94,A18)</f>
+        <f>COUNTIF(Tracker!$L$2:$L$95,A18)</f>
         <v/>
       </c>
     </row>
@@ -6865,7 +6928,7 @@
         </is>
       </c>
       <c r="B19" s="3">
-        <f>COUNTIF(Tracker!$L$2:$L$94,A19)</f>
+        <f>COUNTIF(Tracker!$L$2:$L$95,A19)</f>
         <v/>
       </c>
     </row>
@@ -6876,7 +6939,7 @@
         </is>
       </c>
       <c r="B20" s="3">
-        <f>COUNTIF(Tracker!$L$2:$L$94,A20)</f>
+        <f>COUNTIF(Tracker!$L$2:$L$95,A20)</f>
         <v/>
       </c>
     </row>
@@ -6887,7 +6950,7 @@
         </is>
       </c>
       <c r="B21" s="3">
-        <f>COUNTIF(Tracker!$L$2:$L$94,A21)</f>
+        <f>COUNTIF(Tracker!$L$2:$L$95,A21)</f>
         <v/>
       </c>
     </row>
@@ -6898,7 +6961,7 @@
         </is>
       </c>
       <c r="B22" s="3">
-        <f>COUNTIF(Tracker!$L$2:$L$94,A22)</f>
+        <f>COUNTIF(Tracker!$L$2:$L$95,A22)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Validate S5 bake mechanic; approve Proxie yelp beat
- Received Jeff's source portrait (planning/reference/cats/profileProjection.jpg),
  built a Python/numpy prototype of the bit-plane decomposition
  (scripts/prototypes/bake-projector-image-prototype.py) and confirmed
  the mechanic: partial projector counts genuinely read as noise, the
  face clearly resolves by 3-4 projectors on. Previews committed to
  planning/reference/s5-lightworks/.
- Bumped grid resolution 30x30 -> 60x60 per Jeff's request for a
  stronger likeness (tested 30/45/60/80 side by side; cost is
  negligible either way, tradeoff is purely aesthetic).
- Rubber-hand-illusion yelp comedy beat: APPROVED. Tracker rows updated
  (3 of 7 decisions now resolved).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01398eRPKBRTjBJQ4FDyfbo8
</commit_message>
<xml_diff>
--- a/planning/asset-tracker.xlsx
+++ b/planning/asset-tracker.xlsx
@@ -979,7 +979,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Approve Proxie yelp comedy beat in rubber-hand illusion?</t>
+          <t>RESOLVED — Proxie yelp comedy beat APPROVED</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -1007,12 +1007,12 @@
       <c r="K5" s="6" t="inlineStr"/>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>NEEDS JEFF</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>Fallback: mannequin arm as subject, Proxie narrates.</t>
+          <t>Confirmed 2026-07-19: 'I love that comedy beat! definitely implement it' — build as speced, no mannequin-arm fallback needed.</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>Pickup; tap triggers Proxie flinch+yelp (pending Jeff approval).</t>
+          <t>Pickup; tap triggers Proxie flinch+yelp (APPROVED 2026-07-19).</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
@@ -6281,12 +6281,12 @@
       </c>
       <c r="I88" s="6" t="inlineStr">
         <is>
-          <t>Stroke-zone counting (N&gt;=5) -&gt; Proxie twitch anim; hammer tap -&gt; flinch+yelp; desktop click auto-stroke.</t>
+          <t>Stroke-zone counting (N&gt;=5) -&gt; Proxie twitch anim; hammer tap -&gt; flinch+yelp; desktop click auto-stroke. Yelp beat APPROVED 2026-07-19.</t>
         </is>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>Needs avatar anim states or mannequin-arm fallback — decide by Sat noon.</t>
+          <t>Needs avatar anim states (twitch/flinch) on the Proxie rig once it exists; billboard fallback = a same-named 2-frame flinch sprite swap.</t>
         </is>
       </c>
       <c r="K88" s="6" t="inlineStr">

</xml_diff>

<commit_message>
S5 HUD becomes a real-screenshot carousel, not a composed static image
Jeff supplied 5 actual transparent-PNG captures from the Even Realities
G2 simulator running his real SIGGRAPH 2026 guide app (title, welcome,
starred, sessions, session detail). Redesigned the HUD (TECH_SPEC C.2)
as a texture-swap carousel: click left/right third of the head-locked
panel to page between screens -- reuses the mini-game's screen-third
click pattern instead of adding swipe-gesture detection, so paging costs
zero new systems. Transparent PNGs let the S5 alcove show through around
the UI, matching how a real see-through smart-glasses display works.

WORLD_DESIGNS + tracker updated to match. Blocked on both the reference
render and the 5 captures landing on disk -- Jeff pushing them to
planning/reference/s5-lightworks/.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01398eRPKBRTjBJQ4FDyfbo8
</commit_message>
<xml_diff>
--- a/planning/asset-tracker.xlsx
+++ b/planning/asset-tracker.xlsx
@@ -4400,7 +4400,7 @@
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>Pickup -&gt; green monochrome HUD overlay (real SIGGRAPH 2026 guide app branding, RESOLVED); gaze-glow affordance draws the eye (Jeff's reference render); toggle off.</t>
+          <t>Pickup -&gt; green monochrome HUD carousel of 5 REAL simulator screen captures (title/welcome/starred/sessions/detail, transparent PNG -- scene shows through around the UI); click left/right third of panel pages between them; gaze-glow affordance draws the eye; toggle off.</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr">
@@ -4415,7 +4415,7 @@
       </c>
       <c r="M58" s="6" t="inlineStr">
         <is>
-          <t>Jeff's verbatim ask + reference render received 2026-07-19. #3 in Tripo queue</t>
+          <t>Reference render received; 5 real screen captures pending push (planning/reference/s5-lightworks/hud-captures/). #3 in Tripo queue</t>
         </is>
       </c>
     </row>
@@ -5718,7 +5718,7 @@
       </c>
       <c r="I79" s="6" t="inlineStr">
         <is>
-          <t>TECH_SPEC C.2 — CSS overlay desktop / head-locked 1024x512 CanvasTexture quad XR; green phosphor SIGGRAPH 2026 guide-app content -- REAL branding from Jeff's reference render (wordmark, dates, byline), not placeholder schedule copy; toggle off via re-click/Esc/G.</t>
+          <t>TECH_SPEC C.2 -- head-locked quad (XR) / DOM overlay (desktop), texture-swap carousel across Jeff's 5 REAL simulator screen captures (transparent PNG, no invented content); click-third paging (left=prev, right=next, matches mini-game screen-third pattern); toggle off via re-click/Esc/G.</t>
         </is>
       </c>
       <c r="J79" s="6" t="inlineStr">

</xml_diff>

<commit_message>
S5 HUD carousel: expand to Jeff's actual 9 real screen captures
Pulled Jeff's push (planning/reference/s5-lightworks/hud-captures/) --
9 transparent PNGs, not the 5 originally discussed: loading/title,
welcome, starred, sessions, session detail, speakers, speaker detail,
expo, expo detail. All 576x288 (2:1, matches the panel), ~100KB total.
Numeric filename prefixes give the canonical paging order, so the
carousel design needs no changes beyond the screen list itself.

TECH_SPEC C.2, WORLD_DESIGNS, and the tracker updated to the real
filenames and 9-screen count; glasses-prop tracker row flipped to READY
now that content is fully resolved (only the GLB generation remains).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01398eRPKBRTjBJQ4FDyfbo8
</commit_message>
<xml_diff>
--- a/planning/asset-tracker.xlsx
+++ b/planning/asset-tracker.xlsx
@@ -4400,7 +4400,7 @@
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>Pickup -&gt; green monochrome HUD carousel of 5 REAL simulator screen captures (title/welcome/starred/sessions/detail, transparent PNG -- scene shows through around the UI); click left/right third of panel pages between them; gaze-glow affordance draws the eye; toggle off.</t>
+          <t>Pickup -&gt; green monochrome HUD carousel of 9 REAL simulator screen captures (loading/welcome/starred/sessions/detail/speakers/speaker-detail/expo/expo-detail, transparent PNG -- scene shows through around the UI); click left/right third of panel pages between them; gaze-glow affordance draws the eye; toggle off.</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr">
@@ -4410,12 +4410,12 @@
       </c>
       <c r="L58" s="6" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="M58" s="6" t="inlineStr">
         <is>
-          <t>Reference render received; 5 real screen captures pending push (planning/reference/s5-lightworks/hud-captures/). #3 in Tripo queue</t>
+          <t>Reference render + all 9 real screen captures RECEIVED and committed (planning/reference/s5-lightworks/). #3 in Tripo queue -- glasses GLB itself still to generate</t>
         </is>
       </c>
     </row>
@@ -5718,7 +5718,7 @@
       </c>
       <c r="I79" s="6" t="inlineStr">
         <is>
-          <t>TECH_SPEC C.2 -- head-locked quad (XR) / DOM overlay (desktop), texture-swap carousel across Jeff's 5 REAL simulator screen captures (transparent PNG, no invented content); click-third paging (left=prev, right=next, matches mini-game screen-third pattern); toggle off via re-click/Esc/G.</t>
+          <t>TECH_SPEC C.2 -- head-locked quad (XR) / DOM overlay (desktop), texture-swap carousel across Jeff's 9 REAL simulator screen captures (transparent PNG, no invented content); click-third paging (left=prev, right=next, matches mini-game screen-third pattern); toggle off via re-click/Esc/G.</t>
         </is>
       </c>
       <c r="J79" s="6" t="inlineStr">

</xml_diff>

<commit_message>
S5 NDA pass: approved with one factual correction, guardrail noted
Jeff approved the 'million-dollar hardware' dramatic license as-is. The
'sum wall' placard was fixed: 'bypasses the network entirely' was
factually wrong -- the real optical all-reduce mechanism skips
sequential collect-and-sum, computing the sum in a single parallel step
(Jeff's correction). Also recorded an internal-only guardrail: the
Nature Communications acceptance he mentioned is not on his public site
and stays out of all in-game/public content -- placards and the site
both stay at 'papers pending.' Tracker: NDA decision resolved (4 of 7
walkthrough decisions now done, 3 remain).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01398eRPKBRTjBJQ4FDyfbo8
</commit_message>
<xml_diff>
--- a/planning/asset-tracker.xlsx
+++ b/planning/asset-tracker.xlsx
@@ -1034,7 +1034,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>NDA pass on all S5 placard texts (drafted from public site only)</t>
+          <t>RESOLVED — NDA pass on S5 placard texts: APPROVED with one correction</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1062,12 +1062,12 @@
       <c r="K6" s="6" t="inlineStr"/>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>NEEDS JEFF</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>See WORLD_DESIGNS S5(f).</t>
+          <t>'Million-dollar hardware' line approved as dramatic license (true to how delicate/expensive the real equipment is). 'Sum wall' placard corrected: was 'bypasses the network entirely' (factually wrong) -&gt; now 'skips sequential collect-and-sum, sum appears in a single parallel glance' (Jeff's actual mechanism). GUARDRAIL: do NOT reference the Nature Communications submission anywhere in-game or on placards -- not yet public, still NDA-adjacent per Jeff 2026-07-19; site + placards stay at 'papers pending.'</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reference photos received: data glove, Tobii, mini-game island, Vive, Second Studio
5 files from Jeff (planning/reference/phd research/, planning/reference/
secondstudio/): a labeled data-glove sensor diagram (reveals thumb=jump/
throw and wrist=camera-view-toggle mechanics beyond the gaze+forward-walk
already speced), the Tobii tracker unit, a real screenshot of the PhD
Unity island (rope bridge, torii-style arch, mossy hills), a clean HTC
Vive product shot, and real Second Studio footage showing a mountain-
vista platform -- not the abstract wireframe void currently speced for
S4. Tracker: reference-photos decision resolved; S4 direction flagged
as an open question pending Jeff's call.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01398eRPKBRTjBJQ4FDyfbo8
</commit_message>
<xml_diff>
--- a/planning/asset-tracker.xlsx
+++ b/planning/asset-tracker.xlsx
@@ -1089,7 +1089,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Drop reference photos in reference/ folders: data glove, Vive, G1 glasses, RNLAF era, Prez captures</t>
+          <t>RESOLVED — Reference photos: data glove, Tobii, mini-game island, Vive, Second Studio env RECEIVED</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1117,12 +1117,12 @@
       <c r="K7" s="6" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>NEEDS JEFF</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>Each strong photo converts a risky text-only generation into image-led.</t>
+          <t>planning/reference/phd research/ (dataglove uncovered.jpg -- labeled sensor diagram, unlocks jump/throw/camera-toggle mechanics not yet speced; tobii eyetracker.png; minigame environment.png -- real island screenshot: rope bridge, torii-style wooden arch, mossy hills, sand) and planning/reference/secondstudio/ (htc vive.png -- clean product shot; environment with 3D assets.png -- REAL Second Studio footage: mountain-vista platform, not the abstract wireframe void currently speced -- OPEN QUESTION back to Jeff on which direction for S4). RNLAF-era and Prez captures still welcome if he has them, not blocking.</t>
         </is>
       </c>
     </row>

</xml_diff>